<commit_message>
Adding the latest measures file for this project
</commit_message>
<xml_diff>
--- a/Global_Markets_Pulse_Measures/Global_Index_Overview_Measures.xlsx
+++ b/Global_Markets_Pulse_Measures/Global_Index_Overview_Measures.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E140"/>
+  <dimension ref="A1:E138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4521,7 +4521,7 @@
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>Decimal number, 2 decimals</t>
+          <t>Whole number</t>
         </is>
       </c>
       <c r="E94" s="3" t="inlineStr">
@@ -4884,7 +4884,7 @@
       </c>
       <c r="D100" s="5" t="inlineStr">
         <is>
-          <t>Decimal number (General)</t>
+          <t>Percentage, 2 decimals</t>
         </is>
       </c>
       <c r="E100" s="3" t="inlineStr">
@@ -4977,7 +4977,7 @@
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t>Decimal number (General)</t>
+          <t>Percentage, 2 decimals</t>
         </is>
       </c>
       <c r="E102" s="3" t="inlineStr">
@@ -5553,6 +5553,15 @@
         NOT ISBLANK(
             CALCULATE([Annualized Volatility (Selected Period)])
         )
+            &amp;&amp; NOT ISBLANK(
+                CALCULATE([Maximum Drawdown %])
+            )
+            &amp;&amp; NOT ISBLANK(
+                CALCULATE([CVaR 95%])
+            )
+            &amp;&amp; NOT ISBLANK(
+                CALCULATE([Loss Probability %])
+            )
     )
 VAR NumberOfIndices =
     COUNTROWS(IndexUniverse)
@@ -5563,16 +5572,16 @@
         [Annualized Volatility (Selected Period)],
         ,
         ASC,
-        DENSE
-    )
-/* More negative drawdown = higher risk */
+        SKIP
+    )
+/* More negative maximum drawdown = higher risk */
 VAR DrawdownRank =
     RANKX(
         IndexUniverse,
         [Maximum Drawdown %],
         ,
         DESC,
-        DENSE
+        SKIP
     )
 /* More negative CVaR = higher risk */
 VAR CVaRRank =
@@ -5581,7 +5590,7 @@
         [CVaR 95%],
         ,
         DESC,
-        DENSE
+        SKIP
     )
 /* Higher loss probability = higher risk */
 VAR LossProbabilityRank =
@@ -5590,15 +5599,16 @@
         [Loss Probability %],
         ,
         ASC,
-        DENSE
+        SKIP
     )
 VAR CompositeRank =
-    (
+    DIVIDE(
         VolatilityRank
-        + DrawdownRank
-        + CVaRRank
-        + LossProbabilityRank
-    ) / 4
+            + DrawdownRank
+            + CVaRRank
+            + LossProbabilityRank,
+        4
+    )
 RETURN
     IF(
         NumberOfIndices &gt; 1,
@@ -5616,7 +5626,7 @@
       </c>
       <c r="E113" s="3" t="inlineStr">
         <is>
-          <t>Measure: Risk Score. Creates a relative 0–100 composite risk score across the selected indices using equal-weight rankings of annualized volatility, maximum drawdown, 95% CVaR, and loss probability. Higher scores indicate greater relative risk.</t>
+          <t>Measure: Risk Score. Calculates a relative composite risk score from 0 to 100 across the selected indices using four equally weighted risk dimensions: Annualized Volatility (Selected Period), Maximum Drawdown %, CVaR 95%, and Loss Probability %. Each component is ranked across the selected index universe and the rankings are combined into a normalized score. Higher scores indicate higher relative risk compared with the other selected indices. The score is relative to the current filter context and should not be interpreted as an absolute measure of market risk.</t>
         </is>
       </c>
     </row>
@@ -5671,7 +5681,7 @@
       </c>
       <c r="D115" s="5" t="inlineStr">
         <is>
-          <t>Decimal number (General)</t>
+          <t>Decimal number, 2 decimals</t>
         </is>
       </c>
       <c r="E115" s="3" t="inlineStr">
@@ -5823,7 +5833,7 @@
       </c>
       <c r="D118" s="5" t="inlineStr">
         <is>
-          <t>Decimal number (General)</t>
+          <t>Decimal number, 2 decimals</t>
         </is>
       </c>
       <c r="E118" s="3" t="inlineStr">
@@ -5860,7 +5870,7 @@
       </c>
       <c r="D119" s="5" t="inlineStr">
         <is>
-          <t>Percentage, 2 decimals</t>
+          <t>Decimal number, 2 decimals</t>
         </is>
       </c>
       <c r="E119" s="3" t="inlineStr">
@@ -6019,7 +6029,7 @@
       </c>
     </row>
     <row r="123" ht="345" customHeight="1">
-      <c r="A123" s="6" t="n"/>
+      <c r="A123" s="7" t="n"/>
       <c r="B123" s="3" t="inlineStr">
         <is>
           <t>Risk\Tail Risk</t>
@@ -6061,132 +6071,18 @@
         </is>
       </c>
     </row>
-    <row r="124" ht="400" customHeight="1">
-      <c r="A124" s="6" t="n"/>
+    <row r="124" ht="75" customHeight="1">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
       <c r="B124" s="3" t="inlineStr">
         <is>
-          <t>Risk\Tail Risk</t>
+          <t>KPI\Rankings</t>
         </is>
       </c>
       <c r="C124" s="4" t="inlineStr">
-        <is>
-          <t>VaR Breach Frequency 95% =
-VAR SelectedDates =
-    ALLSELECTED('Calendar'[Date])
-VAR DailyReturnsTable =
-    FILTER(
-        ADDCOLUMNS(
-            SelectedDates,
-            "@DailyReturn",
-                CALCULATE([Daily Return %])
-        ),
-        NOT ISBLANK([@DailyReturn])
-    )
-VAR VaR95 =
-    PERCENTILEX.INC(
-        DailyReturnsTable,
-        [@DailyReturn],
-        0.05
-    )
-VAR BreachDays =
-    COUNTROWS(
-        FILTER(
-            DailyReturnsTable,
-            [@DailyReturn] &lt; VaR95
-        )
-    )
-VAR TotalDays =
-    COUNTROWS(DailyReturnsTable)
-RETURN
-    IF(
-        TotalDays &gt; 0,
-        DIVIDE(
-            BreachDays,
-            TotalDays
-        )
-    )</t>
-        </is>
-      </c>
-      <c r="D124" s="5" t="inlineStr">
-        <is>
-          <t>Percentage, 2 decimals</t>
-        </is>
-      </c>
-      <c r="E124" s="3" t="inlineStr">
-        <is>
-          <t>Measure: VaR Breach Frequency 95%. Calculates the percentage of daily return observations that fall below the historical 95% VaR threshold during the selected period.</t>
-        </is>
-      </c>
-    </row>
-    <row r="125" ht="400" customHeight="1">
-      <c r="A125" s="7" t="n"/>
-      <c r="B125" s="3" t="inlineStr">
-        <is>
-          <t>Risk\Tail Risk</t>
-        </is>
-      </c>
-      <c r="C125" s="4" t="inlineStr">
-        <is>
-          <t>VaR Breach Frequency 99% =
-VAR SelectedDates =
-    ALLSELECTED('Calendar'[Date])
-VAR DailyReturnsTable =
-    FILTER(
-        ADDCOLUMNS(
-            SelectedDates,
-            "@DailyReturn",
-                CALCULATE([Daily Return %])
-        ),
-        NOT ISBLANK([@DailyReturn])
-    )
-VAR VaR99 =
-    PERCENTILEX.INC(
-        DailyReturnsTable,
-        [@DailyReturn],
-        0.01
-    )
-VAR BreachDays =
-    COUNTROWS(
-        FILTER(
-            DailyReturnsTable,
-            [@DailyReturn] &lt; VaR99
-        )
-    )
-VAR TotalDays =
-    COUNTROWS(DailyReturnsTable)
-RETURN
-    IF(
-        TotalDays &gt; 0,
-        DIVIDE(
-            BreachDays,
-            TotalDays
-        )
-    )</t>
-        </is>
-      </c>
-      <c r="D125" s="5" t="inlineStr">
-        <is>
-          <t>Percentage, 2 decimals</t>
-        </is>
-      </c>
-      <c r="E125" s="3" t="inlineStr">
-        <is>
-          <t>Measure: VaR Breach Frequency 99%. Calculates the percentage of daily return observations that fall below the historical 99% VaR threshold during the selected period.</t>
-        </is>
-      </c>
-    </row>
-    <row r="126" ht="75" customHeight="1">
-      <c r="A126" s="2" t="inlineStr">
-        <is>
-          <t>KPI</t>
-        </is>
-      </c>
-      <c r="B126" s="3" t="inlineStr">
-        <is>
-          <t>KPI\Rankings</t>
-        </is>
-      </c>
-      <c r="C126" s="4" t="inlineStr">
         <is>
           <t>Average Market Return % =
 AVERAGEX(
@@ -6195,25 +6091,25 @@
 )</t>
         </is>
       </c>
-      <c r="D126" s="5" t="inlineStr">
-        <is>
-          <t>Percentage, 2 decimals</t>
-        </is>
-      </c>
-      <c r="E126" s="3" t="inlineStr">
+      <c r="D124" s="5" t="inlineStr">
+        <is>
+          <t>Percentage, 2 decimals</t>
+        </is>
+      </c>
+      <c r="E124" s="3" t="inlineStr">
         <is>
           <t>Measure: Average Market Return %. Calculates the average cumulative return across all selected indices in the current filter context.</t>
         </is>
       </c>
     </row>
-    <row r="127" ht="180" customHeight="1">
-      <c r="A127" s="6" t="n"/>
-      <c r="B127" s="3" t="inlineStr">
+    <row r="125" ht="180" customHeight="1">
+      <c r="A125" s="6" t="n"/>
+      <c r="B125" s="3" t="inlineStr">
         <is>
           <t>KPI\Rankings</t>
         </is>
       </c>
-      <c r="C127" s="4" t="inlineStr">
+      <c r="C125" s="4" t="inlineStr">
         <is>
           <t>Best Performer Return % =
 MAXX(
@@ -6229,25 +6125,25 @@
 )</t>
         </is>
       </c>
-      <c r="D127" s="5" t="inlineStr">
-        <is>
-          <t>Percentage, 2 decimals</t>
-        </is>
-      </c>
-      <c r="E127" s="3" t="inlineStr">
+      <c r="D125" s="5" t="inlineStr">
+        <is>
+          <t>Percentage, 2 decimals</t>
+        </is>
+      </c>
+      <c r="E125" s="3" t="inlineStr">
         <is>
           <t>Measure: Best Performer Return %. Returns the cumulative return percentage of the best-performing index in the current filter context.</t>
         </is>
       </c>
     </row>
-    <row r="128" ht="240" customHeight="1">
-      <c r="A128" s="6" t="n"/>
-      <c r="B128" s="3" t="inlineStr">
+    <row r="126" ht="240" customHeight="1">
+      <c r="A126" s="6" t="n"/>
+      <c r="B126" s="3" t="inlineStr">
         <is>
           <t>KPI\Rankings</t>
         </is>
       </c>
-      <c r="C128" s="4" t="inlineStr">
+      <c r="C126" s="4" t="inlineStr">
         <is>
           <t>Best Performing Index =
 VAR TopIndexTable =
@@ -6267,25 +6163,25 @@
     )</t>
         </is>
       </c>
-      <c r="D128" s="5" t="inlineStr">
+      <c r="D126" s="5" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E128" s="3" t="inlineStr">
+      <c r="E126" s="3" t="inlineStr">
         <is>
           <t>Measure: Best Performing Index. Returns the name of the index with the highest cumulative return in the current filter context.</t>
         </is>
       </c>
     </row>
-    <row r="129" ht="240" customHeight="1">
-      <c r="A129" s="6" t="n"/>
-      <c r="B129" s="3" t="inlineStr">
+    <row r="127" ht="240" customHeight="1">
+      <c r="A127" s="6" t="n"/>
+      <c r="B127" s="3" t="inlineStr">
         <is>
           <t>KPI\Rankings</t>
         </is>
       </c>
-      <c r="C129" s="4" t="inlineStr">
+      <c r="C127" s="4" t="inlineStr">
         <is>
           <t>Bottom 3 Performer Flag =
 VAR TotalIndices =
@@ -6303,25 +6199,25 @@
     )</t>
         </is>
       </c>
-      <c r="D129" s="5" t="inlineStr">
+      <c r="D127" s="5" t="inlineStr">
         <is>
           <t>Whole number</t>
         </is>
       </c>
-      <c r="E129" s="3" t="inlineStr">
+      <c r="E127" s="3" t="inlineStr">
         <is>
           <t>Measure: Bottom 3 Performer Flag. Returns 1 when the index is among the bottom three performers based on cumulative return; otherwise returns 0.</t>
         </is>
       </c>
     </row>
-    <row r="130" ht="180" customHeight="1">
-      <c r="A130" s="6" t="n"/>
-      <c r="B130" s="3" t="inlineStr">
+    <row r="128" ht="180" customHeight="1">
+      <c r="A128" s="6" t="n"/>
+      <c r="B128" s="3" t="inlineStr">
         <is>
           <t>KPI\Rankings</t>
         </is>
       </c>
-      <c r="C130" s="4" t="inlineStr">
+      <c r="C128" s="4" t="inlineStr">
         <is>
           <t>Highest Average Volume =
 MAXX(
@@ -6337,25 +6233,25 @@
 )</t>
         </is>
       </c>
-      <c r="D130" s="5" t="inlineStr">
+      <c r="D128" s="5" t="inlineStr">
         <is>
           <t>Whole number</t>
         </is>
       </c>
-      <c r="E130" s="3" t="inlineStr">
+      <c r="E128" s="3" t="inlineStr">
         <is>
           <t>Measure: Highest Average Volume. Returns the highest 30-day average trading volume among the selected indices.</t>
         </is>
       </c>
     </row>
-    <row r="131" ht="240" customHeight="1">
-      <c r="A131" s="6" t="n"/>
-      <c r="B131" s="3" t="inlineStr">
+    <row r="129" ht="240" customHeight="1">
+      <c r="A129" s="6" t="n"/>
+      <c r="B129" s="3" t="inlineStr">
         <is>
           <t>KPI\Rankings</t>
         </is>
       </c>
-      <c r="C131" s="4" t="inlineStr">
+      <c r="C129" s="4" t="inlineStr">
         <is>
           <t>Highest Volume Index =
 VAR TopVolumeTable =
@@ -6375,18 +6271,76 @@
     )</t>
         </is>
       </c>
+      <c r="D129" s="5" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E129" s="3" t="inlineStr">
+        <is>
+          <t>Measure: Highest Volume Index. Returns the name of the index with the highest 30-day average trading volume in the current filter context.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="105" customHeight="1">
+      <c r="A130" s="6" t="n"/>
+      <c r="B130" s="3" t="inlineStr">
+        <is>
+          <t>KPI\Rankings</t>
+        </is>
+      </c>
+      <c r="C130" s="4" t="inlineStr">
+        <is>
+          <t>Number of Outperforming Markets =
+COUNTROWS(
+    FILTER(
+        ALLSELECTED('Dim_Index'[Index]),
+        [Outperforming Market Flag] = 1
+    )
+)</t>
+        </is>
+      </c>
+      <c r="D130" s="5" t="inlineStr">
+        <is>
+          <t>Whole number</t>
+        </is>
+      </c>
+      <c r="E130" s="3" t="inlineStr">
+        <is>
+          <t>Measure: Number of Outperforming Markets. Counts the number of selected indices whose cumulative return is above the average market return.</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="105" customHeight="1">
+      <c r="A131" s="6" t="n"/>
+      <c r="B131" s="3" t="inlineStr">
+        <is>
+          <t>KPI\Rankings</t>
+        </is>
+      </c>
+      <c r="C131" s="4" t="inlineStr">
+        <is>
+          <t>Number of Underperforming Markets =
+COUNTROWS(
+    FILTER(
+        ALLSELECTED('Dim_Index'[Index]),
+        [Outperforming Market Flag] = 0
+    )
+)</t>
+        </is>
+      </c>
       <c r="D131" s="5" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Whole number</t>
         </is>
       </c>
       <c r="E131" s="3" t="inlineStr">
         <is>
-          <t>Measure: Highest Volume Index. Returns the name of the index with the highest 30-day average trading volume in the current filter context.</t>
-        </is>
-      </c>
-    </row>
-    <row r="132" ht="105" customHeight="1">
+          <t>Measure: Number of Underperforming Markets. Counts the number of selected indices whose cumulative return is less than or equal to the average market return.</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="210" customHeight="1">
       <c r="A132" s="6" t="n"/>
       <c r="B132" s="3" t="inlineStr">
         <is>
@@ -6394,64 +6348,6 @@
         </is>
       </c>
       <c r="C132" s="4" t="inlineStr">
-        <is>
-          <t>Number of Outperforming Markets =
-COUNTROWS(
-    FILTER(
-        ALLSELECTED('Dim_Index'[Index]),
-        [Outperforming Market Flag] = 1
-    )
-)</t>
-        </is>
-      </c>
-      <c r="D132" s="5" t="inlineStr">
-        <is>
-          <t>Whole number</t>
-        </is>
-      </c>
-      <c r="E132" s="3" t="inlineStr">
-        <is>
-          <t>Measure: Number of Outperforming Markets. Counts the number of selected indices whose cumulative return is above the average market return.</t>
-        </is>
-      </c>
-    </row>
-    <row r="133" ht="105" customHeight="1">
-      <c r="A133" s="6" t="n"/>
-      <c r="B133" s="3" t="inlineStr">
-        <is>
-          <t>KPI\Rankings</t>
-        </is>
-      </c>
-      <c r="C133" s="4" t="inlineStr">
-        <is>
-          <t>Number of Underperforming Markets =
-COUNTROWS(
-    FILTER(
-        ALLSELECTED('Dim_Index'[Index]),
-        [Outperforming Market Flag] = 0
-    )
-)</t>
-        </is>
-      </c>
-      <c r="D133" s="5" t="inlineStr">
-        <is>
-          <t>Whole number</t>
-        </is>
-      </c>
-      <c r="E133" s="3" t="inlineStr">
-        <is>
-          <t>Measure: Number of Underperforming Markets. Counts the number of selected indices whose cumulative return is less than or equal to the average market return.</t>
-        </is>
-      </c>
-    </row>
-    <row r="134" ht="210" customHeight="1">
-      <c r="A134" s="6" t="n"/>
-      <c r="B134" s="3" t="inlineStr">
-        <is>
-          <t>KPI\Rankings</t>
-        </is>
-      </c>
-      <c r="C134" s="4" t="inlineStr">
         <is>
           <t>Outperforming Market Flag =
 VAR CurrentReturn =
@@ -6467,25 +6363,25 @@
 )</t>
         </is>
       </c>
-      <c r="D134" s="5" t="inlineStr">
+      <c r="D132" s="5" t="inlineStr">
         <is>
           <t>Whole number</t>
         </is>
       </c>
-      <c r="E134" s="3" t="inlineStr">
+      <c r="E132" s="3" t="inlineStr">
         <is>
           <t>Measure: Outperforming Market Flag. Returns 1 when the selected index has a cumulative return greater than the average cumulative return of all selected indices.</t>
         </is>
       </c>
     </row>
-    <row r="135" ht="225" customHeight="1">
-      <c r="A135" s="6" t="n"/>
-      <c r="B135" s="3" t="inlineStr">
+    <row r="133" ht="225" customHeight="1">
+      <c r="A133" s="6" t="n"/>
+      <c r="B133" s="3" t="inlineStr">
         <is>
           <t>KPI\Rankings</t>
         </is>
       </c>
-      <c r="C135" s="4" t="inlineStr">
+      <c r="C133" s="4" t="inlineStr">
         <is>
           <t>Performance Rank =
 VAR CurrentReturn =
@@ -6503,25 +6399,25 @@
     )</t>
         </is>
       </c>
-      <c r="D135" s="5" t="inlineStr">
+      <c r="D133" s="5" t="inlineStr">
         <is>
           <t>Whole number</t>
         </is>
       </c>
-      <c r="E135" s="3" t="inlineStr">
+      <c r="E133" s="3" t="inlineStr">
         <is>
           <t>Measure: Performance Rank. Ranks the selected indices from highest to lowest based on cumulative return during the selected date period.</t>
         </is>
       </c>
     </row>
-    <row r="136" ht="285" customHeight="1">
-      <c r="A136" s="6" t="n"/>
-      <c r="B136" s="3" t="inlineStr">
+    <row r="134" ht="285" customHeight="1">
+      <c r="A134" s="6" t="n"/>
+      <c r="B134" s="3" t="inlineStr">
         <is>
           <t>KPI\Rankings</t>
         </is>
       </c>
-      <c r="C136" s="4" t="inlineStr">
+      <c r="C134" s="4" t="inlineStr">
         <is>
           <t>Performance Spread % =
 VAR BestReturn =
@@ -6542,25 +6438,25 @@
     )</t>
         </is>
       </c>
-      <c r="D136" s="5" t="inlineStr">
-        <is>
-          <t>Percentage, 2 decimals</t>
-        </is>
-      </c>
-      <c r="E136" s="3" t="inlineStr">
+      <c r="D134" s="5" t="inlineStr">
+        <is>
+          <t>Percentage, 2 decimals</t>
+        </is>
+      </c>
+      <c r="E134" s="3" t="inlineStr">
         <is>
           <t>Measure: Performance Spread %. Calculates the difference between the highest and lowest cumulative returns among the selected indices.</t>
         </is>
       </c>
     </row>
-    <row r="137" ht="165" customHeight="1">
-      <c r="A137" s="6" t="n"/>
-      <c r="B137" s="3" t="inlineStr">
+    <row r="135" ht="165" customHeight="1">
+      <c r="A135" s="6" t="n"/>
+      <c r="B135" s="3" t="inlineStr">
         <is>
           <t>KPI\Rankings</t>
         </is>
       </c>
-      <c r="C137" s="4" t="inlineStr">
+      <c r="C135" s="4" t="inlineStr">
         <is>
           <t>Top 3 Performer Flag =
 VAR CurrentRank =
@@ -6574,25 +6470,25 @@
     )</t>
         </is>
       </c>
-      <c r="D137" s="5" t="inlineStr">
+      <c r="D135" s="5" t="inlineStr">
         <is>
           <t>Whole number</t>
         </is>
       </c>
-      <c r="E137" s="3" t="inlineStr">
+      <c r="E135" s="3" t="inlineStr">
         <is>
           <t>Measure: Top 3 Performer Flag. Returns 1 when the index is among the top three performers based on cumulative return; otherwise returns 0.</t>
         </is>
       </c>
     </row>
-    <row r="138" ht="225" customHeight="1">
-      <c r="A138" s="6" t="n"/>
-      <c r="B138" s="3" t="inlineStr">
+    <row r="136" ht="225" customHeight="1">
+      <c r="A136" s="6" t="n"/>
+      <c r="B136" s="3" t="inlineStr">
         <is>
           <t>KPI\Rankings</t>
         </is>
       </c>
-      <c r="C138" s="4" t="inlineStr">
+      <c r="C136" s="4" t="inlineStr">
         <is>
           <t>Volume Rank =
 VAR CurrentVolume =
@@ -6610,25 +6506,25 @@
     )</t>
         </is>
       </c>
-      <c r="D138" s="5" t="inlineStr">
+      <c r="D136" s="5" t="inlineStr">
         <is>
           <t>Whole number</t>
         </is>
       </c>
-      <c r="E138" s="3" t="inlineStr">
+      <c r="E136" s="3" t="inlineStr">
         <is>
           <t>Measure: Volume Rank. Ranks the selected indices from highest to lowest based on their 30-day average trading volume.</t>
         </is>
       </c>
     </row>
-    <row r="139" ht="180" customHeight="1">
-      <c r="A139" s="6" t="n"/>
-      <c r="B139" s="3" t="inlineStr">
+    <row r="137" ht="180" customHeight="1">
+      <c r="A137" s="6" t="n"/>
+      <c r="B137" s="3" t="inlineStr">
         <is>
           <t>KPI\Rankings</t>
         </is>
       </c>
-      <c r="C139" s="4" t="inlineStr">
+      <c r="C137" s="4" t="inlineStr">
         <is>
           <t>Worst Performer Return % =
 MINX(
@@ -6644,25 +6540,25 @@
 )</t>
         </is>
       </c>
-      <c r="D139" s="5" t="inlineStr">
-        <is>
-          <t>Percentage, 2 decimals</t>
-        </is>
-      </c>
-      <c r="E139" s="3" t="inlineStr">
+      <c r="D137" s="5" t="inlineStr">
+        <is>
+          <t>Percentage, 2 decimals</t>
+        </is>
+      </c>
+      <c r="E137" s="3" t="inlineStr">
         <is>
           <t>Measure: Worst Performer Return %. Returns the cumulative return percentage of the worst-performing index in the current filter context.</t>
         </is>
       </c>
     </row>
-    <row r="140" ht="240" customHeight="1">
-      <c r="A140" s="7" t="n"/>
-      <c r="B140" s="3" t="inlineStr">
+    <row r="138" ht="240" customHeight="1">
+      <c r="A138" s="7" t="n"/>
+      <c r="B138" s="3" t="inlineStr">
         <is>
           <t>KPI\Rankings</t>
         </is>
       </c>
-      <c r="C140" s="4" t="inlineStr">
+      <c r="C138" s="4" t="inlineStr">
         <is>
           <t>Worst Performing Index =
 VAR BottomIndexTable =
@@ -6682,12 +6578,12 @@
     )</t>
         </is>
       </c>
-      <c r="D140" s="5" t="inlineStr">
+      <c r="D138" s="5" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="E140" s="3" t="inlineStr">
+      <c r="E138" s="3" t="inlineStr">
         <is>
           <t>Measure: Worst Performing Index. Returns the name of the index with the lowest cumulative return in the current filter context.</t>
         </is>
@@ -6696,9 +6592,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A2:A15"/>
+    <mergeCell ref="A124:A138"/>
     <mergeCell ref="A16:A92"/>
-    <mergeCell ref="A93:A125"/>
-    <mergeCell ref="A126:A140"/>
+    <mergeCell ref="A93:A123"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10668,7 +10564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -10837,7 +10733,7 @@
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>Decimal number, 2 decimals</t>
+          <t>Whole number</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -11200,7 +11096,7 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Decimal number (General)</t>
+          <t>Percentage, 2 decimals</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -11293,7 +11189,7 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Decimal number (General)</t>
+          <t>Percentage, 2 decimals</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -11869,6 +11765,15 @@
         NOT ISBLANK(
             CALCULATE([Annualized Volatility (Selected Period)])
         )
+            &amp;&amp; NOT ISBLANK(
+                CALCULATE([Maximum Drawdown %])
+            )
+            &amp;&amp; NOT ISBLANK(
+                CALCULATE([CVaR 95%])
+            )
+            &amp;&amp; NOT ISBLANK(
+                CALCULATE([Loss Probability %])
+            )
     )
 VAR NumberOfIndices =
     COUNTROWS(IndexUniverse)
@@ -11879,16 +11784,16 @@
         [Annualized Volatility (Selected Period)],
         ,
         ASC,
-        DENSE
-    )
-/* More negative drawdown = higher risk */
+        SKIP
+    )
+/* More negative maximum drawdown = higher risk */
 VAR DrawdownRank =
     RANKX(
         IndexUniverse,
         [Maximum Drawdown %],
         ,
         DESC,
-        DENSE
+        SKIP
     )
 /* More negative CVaR = higher risk */
 VAR CVaRRank =
@@ -11897,7 +11802,7 @@
         [CVaR 95%],
         ,
         DESC,
-        DENSE
+        SKIP
     )
 /* Higher loss probability = higher risk */
 VAR LossProbabilityRank =
@@ -11906,15 +11811,16 @@
         [Loss Probability %],
         ,
         ASC,
-        DENSE
+        SKIP
     )
 VAR CompositeRank =
-    (
+    DIVIDE(
         VolatilityRank
-        + DrawdownRank
-        + CVaRRank
-        + LossProbabilityRank
-    ) / 4
+            + DrawdownRank
+            + CVaRRank
+            + LossProbabilityRank,
+        4
+    )
 RETURN
     IF(
         NumberOfIndices &gt; 1,
@@ -11932,7 +11838,7 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Measure: Risk Score. Creates a relative 0–100 composite risk score across the selected indices using equal-weight rankings of annualized volatility, maximum drawdown, 95% CVaR, and loss probability. Higher scores indicate greater relative risk.</t>
+          <t>Measure: Risk Score. Calculates a relative composite risk score from 0 to 100 across the selected indices using four equally weighted risk dimensions: Annualized Volatility (Selected Period), Maximum Drawdown %, CVaR 95%, and Loss Probability %. Each component is ranked across the selected index universe and the rankings are combined into a normalized score. Higher scores indicate higher relative risk compared with the other selected indices. The score is relative to the current filter context and should not be interpreted as an absolute measure of market risk.</t>
         </is>
       </c>
     </row>
@@ -11987,7 +11893,7 @@
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Decimal number (General)</t>
+          <t>Decimal number, 2 decimals</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
@@ -12139,7 +12045,7 @@
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Decimal number (General)</t>
+          <t>Decimal number, 2 decimals</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
@@ -12176,7 +12082,7 @@
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Percentage, 2 decimals</t>
+          <t>Decimal number, 2 decimals</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
@@ -12335,7 +12241,7 @@
       </c>
     </row>
     <row r="32" ht="345" customHeight="1">
-      <c r="A32" s="6" t="n"/>
+      <c r="A32" s="7" t="n"/>
       <c r="B32" s="3" t="inlineStr">
         <is>
           <t>Risk\Tail Risk</t>
@@ -12377,123 +12283,9 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="400" customHeight="1">
-      <c r="A33" s="6" t="n"/>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>Risk\Tail Risk</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>VaR Breach Frequency 95% =
-VAR SelectedDates =
-    ALLSELECTED('Calendar'[Date])
-VAR DailyReturnsTable =
-    FILTER(
-        ADDCOLUMNS(
-            SelectedDates,
-            "@DailyReturn",
-                CALCULATE([Daily Return %])
-        ),
-        NOT ISBLANK([@DailyReturn])
-    )
-VAR VaR95 =
-    PERCENTILEX.INC(
-        DailyReturnsTable,
-        [@DailyReturn],
-        0.05
-    )
-VAR BreachDays =
-    COUNTROWS(
-        FILTER(
-            DailyReturnsTable,
-            [@DailyReturn] &lt; VaR95
-        )
-    )
-VAR TotalDays =
-    COUNTROWS(DailyReturnsTable)
-RETURN
-    IF(
-        TotalDays &gt; 0,
-        DIVIDE(
-            BreachDays,
-            TotalDays
-        )
-    )</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>Percentage, 2 decimals</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="inlineStr">
-        <is>
-          <t>Measure: VaR Breach Frequency 95%. Calculates the percentage of daily return observations that fall below the historical 95% VaR threshold during the selected period.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="400" customHeight="1">
-      <c r="A34" s="7" t="n"/>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>Risk\Tail Risk</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>VaR Breach Frequency 99% =
-VAR SelectedDates =
-    ALLSELECTED('Calendar'[Date])
-VAR DailyReturnsTable =
-    FILTER(
-        ADDCOLUMNS(
-            SelectedDates,
-            "@DailyReturn",
-                CALCULATE([Daily Return %])
-        ),
-        NOT ISBLANK([@DailyReturn])
-    )
-VAR VaR99 =
-    PERCENTILEX.INC(
-        DailyReturnsTable,
-        [@DailyReturn],
-        0.01
-    )
-VAR BreachDays =
-    COUNTROWS(
-        FILTER(
-            DailyReturnsTable,
-            [@DailyReturn] &lt; VaR99
-        )
-    )
-VAR TotalDays =
-    COUNTROWS(DailyReturnsTable)
-RETURN
-    IF(
-        TotalDays &gt; 0,
-        DIVIDE(
-            BreachDays,
-            TotalDays
-        )
-    )</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>Percentage, 2 decimals</t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="inlineStr">
-        <is>
-          <t>Measure: VaR Breach Frequency 99%. Calculates the percentage of daily return observations that fall below the historical 99% VaR threshold during the selected period.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:A34"/>
+    <mergeCell ref="A2:A32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>